<commit_message>
Move % Under Target to column B in Good Prices, update MEMORY.md
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/Vortex Matches/output/1130895_Good Prices.xlsx
+++ b/Trading Analysis/Vortex Matches/output/1130895_Good Prices.xlsx
@@ -16,6 +16,9 @@
     <t>RFQ Number</t>
   </si>
   <si>
+    <t>% Under Target</t>
+  </si>
+  <si>
     <t>RFQ Created</t>
   </si>
   <si>
@@ -50,9 +53,6 @@
   </si>
   <si>
     <t>Supplier Price</t>
-  </si>
-  <si>
-    <t>% Under Target</t>
   </si>
   <si>
     <t>lead_time</t>
@@ -304,16 +304,16 @@
   </cellStyleXfs>
   <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="10" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -659,22 +659,22 @@
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="14" style="1" customWidth="1"/>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="12" style="2" customWidth="1"/>
-    <col min="6" max="6" width="14" style="3" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="8" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="22" customWidth="1"/>
-    <col min="11" max="11" width="28" customWidth="1"/>
-    <col min="12" max="12" width="12" style="2" customWidth="1"/>
-    <col min="13" max="13" width="14" style="3" customWidth="1"/>
+    <col min="3" max="3" width="14" style="2" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="12" style="3" customWidth="1"/>
+    <col min="7" max="7" width="14" style="4" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="8" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
+    <col min="11" max="11" width="22" customWidth="1"/>
+    <col min="12" max="12" width="28" customWidth="1"/>
+    <col min="13" max="13" width="12" style="3" customWidth="1"/>
     <col min="14" max="14" width="14" style="4" customWidth="1"/>
     <col min="15" max="16" width="14" customWidth="1"/>
-    <col min="17" max="17" width="14" style="1" customWidth="1"/>
-    <col min="18" max="18" width="20" style="2" customWidth="1"/>
-    <col min="19" max="19" width="14" style="4" customWidth="1"/>
+    <col min="17" max="17" width="14" style="2" customWidth="1"/>
+    <col min="18" max="18" width="20" style="3" customWidth="1"/>
+    <col min="19" max="19" width="14" style="1" customWidth="1"/>
     <col min="20" max="20" width="14" style="5" customWidth="1"/>
   </cols>
   <sheetData>
@@ -685,19 +685,19 @@
       <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="10" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="6" t="s">
@@ -712,7 +712,7 @@
       <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
       <c r="M1" s="9" t="s">
@@ -727,13 +727,13 @@
       <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="7" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="11" t="s">
@@ -745,43 +745,43 @@
         <v>20</v>
       </c>
       <c r="B2" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
+        <v>0.30317324185248706</v>
+      </c>
+      <c r="C2" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
         <v>22</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="3">
         <v>72500</v>
       </c>
-      <c r="F2" s="3">
+      <c r="G2" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G2" t="s">
-        <v>23</v>
-      </c>
       <c r="H2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
         <v>24</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>25</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>22</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>26</v>
       </c>
-      <c r="L2" s="2">
+      <c r="M2" s="3">
         <v>10000</v>
       </c>
-      <c r="M2" s="3">
+      <c r="N2" s="4">
         <v>0.39</v>
-      </c>
-      <c r="N2" s="4">
-        <v>0.30317324185248706</v>
       </c>
       <c r="O2" t="s">
         <v>27</v>
@@ -789,13 +789,13 @@
       <c r="P2" t="s">
         <v>28</v>
       </c>
-      <c r="Q2" s="1">
+      <c r="Q2" s="2">
         <v>46057.94688554398</v>
       </c>
-      <c r="R2" s="2">
+      <c r="R2" s="3">
         <v>33</v>
       </c>
-      <c r="S2" s="4">
+      <c r="S2" s="1">
         <v>0.13793103448275862</v>
       </c>
       <c r="T2" s="5">
@@ -807,43 +807,43 @@
         <v>20</v>
       </c>
       <c r="B3" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
+        <v>0.35677530017152653</v>
+      </c>
+      <c r="C3" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="3">
         <v>72500</v>
       </c>
-      <c r="F3" s="3">
+      <c r="G3" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G3" t="s">
-        <v>23</v>
-      </c>
       <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
         <v>24</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>25</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>22</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="2">
+      <c r="M3" s="3">
         <v>10000</v>
       </c>
-      <c r="M3" s="3">
+      <c r="N3" s="4">
         <v>0.36</v>
-      </c>
-      <c r="N3" s="4">
-        <v>0.35677530017152653</v>
       </c>
       <c r="O3" t="s">
         <v>27</v>
@@ -851,13 +851,13 @@
       <c r="P3" t="s">
         <v>28</v>
       </c>
-      <c r="Q3" s="1">
+      <c r="Q3" s="2">
         <v>46057.20823052083</v>
       </c>
-      <c r="R3" s="2">
+      <c r="R3" s="3">
         <v>33</v>
       </c>
-      <c r="S3" s="4">
+      <c r="S3" s="1">
         <v>0.13793103448275862</v>
       </c>
       <c r="T3" s="5">
@@ -869,43 +869,43 @@
         <v>20</v>
       </c>
       <c r="B4" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
+        <v>0.4461120640365923</v>
+      </c>
+      <c r="C4" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="2">
+      <c r="F4" s="3">
         <v>72500</v>
       </c>
-      <c r="F4" s="3">
+      <c r="G4" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
       <c r="H4" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" t="s">
         <v>24</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>25</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>22</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>26</v>
       </c>
-      <c r="L4" s="2">
+      <c r="M4" s="3">
         <v>50000</v>
       </c>
-      <c r="M4" s="3">
+      <c r="N4" s="4">
         <v>0.31</v>
-      </c>
-      <c r="N4" s="4">
-        <v>0.4461120640365923</v>
       </c>
       <c r="O4" t="s">
         <v>30</v>
@@ -913,13 +913,13 @@
       <c r="P4" t="s">
         <v>31</v>
       </c>
-      <c r="Q4" s="1">
+      <c r="Q4" s="2">
         <v>46027.21528875</v>
       </c>
-      <c r="R4" s="2">
+      <c r="R4" s="3">
         <v>63</v>
       </c>
-      <c r="S4" s="4">
+      <c r="S4" s="1">
         <v>0.6896551724137931</v>
       </c>
       <c r="T4" s="5">
@@ -931,43 +931,43 @@
         <v>20</v>
       </c>
       <c r="B5" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
+        <v>0.48184676958261863</v>
+      </c>
+      <c r="C5" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D5" t="s">
+        <v>21</v>
+      </c>
+      <c r="E5" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="2">
+      <c r="F5" s="3">
         <v>72500</v>
       </c>
-      <c r="F5" s="3">
+      <c r="G5" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G5" t="s">
-        <v>23</v>
-      </c>
       <c r="H5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I5" t="s">
         <v>24</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>25</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>22</v>
       </c>
-      <c r="K5" t="s">
+      <c r="L5" t="s">
         <v>29</v>
       </c>
-      <c r="L5" s="2">
+      <c r="M5" s="3">
         <v>0</v>
       </c>
-      <c r="M5" s="3">
+      <c r="N5" s="4">
         <v>0.29</v>
-      </c>
-      <c r="N5" s="4">
-        <v>0.48184676958261863</v>
       </c>
       <c r="O5" t="s">
         <v>30</v>
@@ -975,13 +975,13 @@
       <c r="P5" t="s">
         <v>23</v>
       </c>
-      <c r="Q5" s="1">
+      <c r="Q5" s="2">
         <v>46026.95746363426</v>
       </c>
-      <c r="R5" s="2">
+      <c r="R5" s="3">
         <v>64</v>
       </c>
-      <c r="S5" s="4">
+      <c r="S5" s="1">
         <v>0</v>
       </c>
       <c r="T5" s="5">
@@ -993,43 +993,43 @@
         <v>20</v>
       </c>
       <c r="B6" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
+        <v>0.7672253258845437</v>
+      </c>
+      <c r="C6" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D6" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="2">
+      <c r="F6" s="3">
         <v>5000</v>
       </c>
-      <c r="F6" s="3">
+      <c r="G6" s="4">
         <v>0.94512</v>
       </c>
-      <c r="G6" t="s">
-        <v>23</v>
-      </c>
       <c r="H6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I6" t="s">
         <v>24</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>25</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
         <v>32</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>29</v>
       </c>
-      <c r="L6" s="2">
+      <c r="M6" s="3">
         <v>50000</v>
       </c>
-      <c r="M6" s="3">
+      <c r="N6" s="4">
         <v>0.22</v>
-      </c>
-      <c r="N6" s="4">
-        <v>0.7672253258845437</v>
       </c>
       <c r="O6" t="s">
         <v>33</v>
@@ -1037,13 +1037,13 @@
       <c r="P6" t="s">
         <v>31</v>
       </c>
-      <c r="Q6" s="1">
+      <c r="Q6" s="2">
         <v>46001.22178418982</v>
       </c>
-      <c r="R6" s="2">
+      <c r="R6" s="3">
         <v>89</v>
       </c>
-      <c r="S6" s="4">
+      <c r="S6" s="1">
         <v>10</v>
       </c>
       <c r="T6" s="5">
@@ -1055,43 +1055,43 @@
         <v>20</v>
       </c>
       <c r="B7" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
+        <v>0.32359307359307354</v>
+      </c>
+      <c r="C7" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s">
         <v>34</v>
       </c>
-      <c r="E7" s="2">
+      <c r="F7" s="3">
         <v>24000</v>
       </c>
-      <c r="F7" s="3">
+      <c r="G7" s="4">
         <v>0.07392</v>
       </c>
-      <c r="G7" t="s">
-        <v>23</v>
-      </c>
       <c r="H7" t="s">
+        <v>23</v>
+      </c>
+      <c r="I7" t="s">
         <v>35</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>36</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
         <v>34</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>37</v>
       </c>
-      <c r="L7" s="2">
+      <c r="M7" s="3">
         <v>1906</v>
       </c>
-      <c r="M7" s="3">
+      <c r="N7" s="4">
         <v>0.05</v>
-      </c>
-      <c r="N7" s="4">
-        <v>0.32359307359307354</v>
       </c>
       <c r="O7" t="s">
         <v>38</v>
@@ -1099,13 +1099,13 @@
       <c r="P7" t="s">
         <v>39</v>
       </c>
-      <c r="Q7" s="1">
+      <c r="Q7" s="2">
         <v>46086.37278019676</v>
       </c>
-      <c r="R7" s="2">
+      <c r="R7" s="3">
         <v>4</v>
       </c>
-      <c r="S7" s="4">
+      <c r="S7" s="1">
         <v>0.07941666666666666</v>
       </c>
       <c r="T7" s="5">
@@ -1117,43 +1117,43 @@
         <v>20</v>
       </c>
       <c r="B8" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
+        <v>0.39123376623376627</v>
+      </c>
+      <c r="C8" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
         <v>40</v>
       </c>
-      <c r="E8" s="2">
+      <c r="F8" s="3">
         <v>24000</v>
       </c>
-      <c r="F8" s="3">
+      <c r="G8" s="4">
         <v>0.07392</v>
       </c>
-      <c r="G8" t="s">
-        <v>23</v>
-      </c>
       <c r="H8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I8" t="s">
         <v>35</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>41</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>40</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>42</v>
       </c>
-      <c r="L8" s="2">
+      <c r="M8" s="3">
         <v>14400</v>
       </c>
-      <c r="M8" s="3">
+      <c r="N8" s="4">
         <v>0.045</v>
-      </c>
-      <c r="N8" s="4">
-        <v>0.39123376623376627</v>
       </c>
       <c r="O8" t="s">
         <v>38</v>
@@ -1161,13 +1161,13 @@
       <c r="P8" t="s">
         <v>43</v>
       </c>
-      <c r="Q8" s="1">
+      <c r="Q8" s="2">
         <v>46086.355969791664</v>
       </c>
-      <c r="R8" s="2">
+      <c r="R8" s="3">
         <v>4</v>
       </c>
-      <c r="S8" s="4">
+      <c r="S8" s="1">
         <v>0.6</v>
       </c>
       <c r="T8" s="5">
@@ -1179,43 +1179,43 @@
         <v>20</v>
       </c>
       <c r="B9" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
+        <v>0.053030303030302935</v>
+      </c>
+      <c r="C9" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D9" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="2">
+      <c r="F9" s="3">
         <v>24000</v>
       </c>
-      <c r="F9" s="3">
+      <c r="G9" s="4">
         <v>0.07392</v>
       </c>
-      <c r="G9" t="s">
-        <v>23</v>
-      </c>
       <c r="H9" t="s">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s">
         <v>35</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>44</v>
       </c>
-      <c r="J9" t="s">
+      <c r="K9" t="s">
         <v>40</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>45</v>
       </c>
-      <c r="L9" s="2">
+      <c r="M9" s="3">
         <v>346</v>
       </c>
-      <c r="M9" s="3">
+      <c r="N9" s="4">
         <v>0.07</v>
-      </c>
-      <c r="N9" s="4">
-        <v>0.053030303030302935</v>
       </c>
       <c r="O9" t="s">
         <v>38</v>
@@ -1223,13 +1223,13 @@
       <c r="P9" t="s">
         <v>23</v>
       </c>
-      <c r="Q9" s="1">
+      <c r="Q9" s="2">
         <v>46086.3559596875</v>
       </c>
-      <c r="R9" s="2">
+      <c r="R9" s="3">
         <v>4</v>
       </c>
-      <c r="S9" s="4">
+      <c r="S9" s="1">
         <v>0.014416666666666666</v>
       </c>
       <c r="T9" s="5">
@@ -1241,43 +1241,43 @@
         <v>20</v>
       </c>
       <c r="B10" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
+        <v>0.5941558441558442</v>
+      </c>
+      <c r="C10" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D10" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="2">
+      <c r="F10" s="3">
         <v>24000</v>
       </c>
-      <c r="F10" s="3">
+      <c r="G10" s="4">
         <v>0.07392</v>
       </c>
-      <c r="G10" t="s">
-        <v>23</v>
-      </c>
       <c r="H10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I10" t="s">
         <v>35</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>36</v>
       </c>
-      <c r="J10" t="s">
+      <c r="K10" t="s">
         <v>34</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="2">
+      <c r="M10" s="3">
         <v>5677</v>
       </c>
-      <c r="M10" s="3">
+      <c r="N10" s="4">
         <v>0.03</v>
-      </c>
-      <c r="N10" s="4">
-        <v>0.5941558441558442</v>
       </c>
       <c r="O10" t="s">
         <v>38</v>
@@ -1285,13 +1285,13 @@
       <c r="P10" t="s">
         <v>47</v>
       </c>
-      <c r="Q10" s="1">
+      <c r="Q10" s="2">
         <v>46086.35546523148</v>
       </c>
-      <c r="R10" s="2">
+      <c r="R10" s="3">
         <v>4</v>
       </c>
-      <c r="S10" s="4">
+      <c r="S10" s="1">
         <v>0.23654166666666668</v>
       </c>
       <c r="T10" s="5">
@@ -1303,43 +1303,43 @@
         <v>20</v>
       </c>
       <c r="B11" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
+        <v>-0.09017921112104338</v>
+      </c>
+      <c r="C11" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D11" t="s">
+        <v>21</v>
+      </c>
+      <c r="E11" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="2">
+      <c r="F11" s="3">
         <v>3382</v>
       </c>
-      <c r="F11" s="3">
+      <c r="G11" s="4">
         <v>0.008228005</v>
       </c>
-      <c r="G11" t="s">
-        <v>23</v>
-      </c>
       <c r="H11" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" t="s">
         <v>35</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>49</v>
       </c>
-      <c r="J11" t="s">
+      <c r="K11" t="s">
         <v>48</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>50</v>
       </c>
-      <c r="L11" s="2">
+      <c r="M11" s="3">
         <v>8000</v>
       </c>
-      <c r="M11" s="3">
+      <c r="N11" s="4">
         <v>0.00897</v>
-      </c>
-      <c r="N11" s="4">
-        <v>-0.09017921112104338</v>
       </c>
       <c r="O11" t="s">
         <v>38</v>
@@ -1347,13 +1347,13 @@
       <c r="P11" t="s">
         <v>51</v>
       </c>
-      <c r="Q11" s="1">
+      <c r="Q11" s="2">
         <v>46086.3509090625</v>
       </c>
-      <c r="R11" s="2">
+      <c r="R11" s="3">
         <v>4</v>
       </c>
-      <c r="S11" s="4">
+      <c r="S11" s="1">
         <v>2.365464222353637</v>
       </c>
       <c r="T11" s="5">
@@ -1365,43 +1365,43 @@
         <v>20</v>
       </c>
       <c r="B12" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C12" t="s">
-        <v>21</v>
+        <v>-0.13636363636363627</v>
+      </c>
+      <c r="C12" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" t="s">
         <v>52</v>
       </c>
-      <c r="E12" s="2">
+      <c r="F12" s="3">
         <v>84000</v>
       </c>
-      <c r="F12" s="3">
+      <c r="G12" s="4">
         <v>4.224</v>
       </c>
-      <c r="G12" t="s">
-        <v>23</v>
-      </c>
       <c r="H12" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" t="s">
         <v>35</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>53</v>
       </c>
-      <c r="J12" t="s">
+      <c r="K12" t="s">
         <v>52</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>54</v>
       </c>
-      <c r="L12" s="2">
+      <c r="M12" s="3">
         <v>84000</v>
       </c>
-      <c r="M12" s="3">
+      <c r="N12" s="4">
         <v>4.8</v>
-      </c>
-      <c r="N12" s="4">
-        <v>-0.13636363636363627</v>
       </c>
       <c r="O12" t="s">
         <v>23</v>
@@ -1409,13 +1409,13 @@
       <c r="P12" t="s">
         <v>55</v>
       </c>
-      <c r="Q12" s="1">
+      <c r="Q12" s="2">
         <v>46085.228698402774</v>
       </c>
-      <c r="R12" s="2">
+      <c r="R12" s="3">
         <v>5</v>
       </c>
-      <c r="S12" s="4">
+      <c r="S12" s="1">
         <v>1</v>
       </c>
       <c r="T12" s="5">
@@ -1427,43 +1427,43 @@
         <v>20</v>
       </c>
       <c r="B13" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C13" t="s">
-        <v>21</v>
+        <v>0.005681818181818186</v>
+      </c>
+      <c r="C13" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D13" t="s">
+        <v>21</v>
+      </c>
+      <c r="E13" t="s">
         <v>52</v>
       </c>
-      <c r="E13" s="2">
+      <c r="F13" s="3">
         <v>84000</v>
       </c>
-      <c r="F13" s="3">
+      <c r="G13" s="4">
         <v>4.224</v>
       </c>
-      <c r="G13" t="s">
-        <v>23</v>
-      </c>
       <c r="H13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" t="s">
         <v>35</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>53</v>
       </c>
-      <c r="J13" t="s">
+      <c r="K13" t="s">
         <v>52</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>54</v>
       </c>
-      <c r="L13" s="2">
+      <c r="M13" s="3">
         <v>30000</v>
       </c>
-      <c r="M13" s="3">
+      <c r="N13" s="4">
         <v>4.2</v>
-      </c>
-      <c r="N13" s="4">
-        <v>0.005681818181818186</v>
       </c>
       <c r="O13" t="s">
         <v>23</v>
@@ -1471,13 +1471,13 @@
       <c r="P13" t="s">
         <v>56</v>
       </c>
-      <c r="Q13" s="1">
+      <c r="Q13" s="2">
         <v>46058.222427824076</v>
       </c>
-      <c r="R13" s="2">
+      <c r="R13" s="3">
         <v>32</v>
       </c>
-      <c r="S13" s="4">
+      <c r="S13" s="1">
         <v>0.35714285714285715</v>
       </c>
       <c r="T13" s="5">
@@ -1489,43 +1489,43 @@
         <v>20</v>
       </c>
       <c r="B14" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C14" t="s">
-        <v>21</v>
+        <v>0.37821612349914235</v>
+      </c>
+      <c r="C14" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D14" t="s">
+        <v>21</v>
+      </c>
+      <c r="E14" t="s">
         <v>22</v>
       </c>
-      <c r="E14" s="2">
+      <c r="F14" s="3">
         <v>72500</v>
       </c>
-      <c r="F14" s="3">
+      <c r="G14" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G14" t="s">
-        <v>23</v>
-      </c>
       <c r="H14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" t="s">
         <v>35</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>44</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>22</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>57</v>
       </c>
-      <c r="L14" s="2">
+      <c r="M14" s="3">
         <v>27500</v>
       </c>
-      <c r="M14" s="3">
+      <c r="N14" s="4">
         <v>0.348</v>
-      </c>
-      <c r="N14" s="4">
-        <v>0.37821612349914235</v>
       </c>
       <c r="O14" t="s">
         <v>58</v>
@@ -1533,13 +1533,13 @@
       <c r="P14" t="s">
         <v>28</v>
       </c>
-      <c r="Q14" s="1">
+      <c r="Q14" s="2">
         <v>46045.12806503472</v>
       </c>
-      <c r="R14" s="2">
+      <c r="R14" s="3">
         <v>45</v>
       </c>
-      <c r="S14" s="4">
+      <c r="S14" s="1">
         <v>0.3793103448275862</v>
       </c>
       <c r="T14" s="5">
@@ -1551,43 +1551,43 @@
         <v>20</v>
       </c>
       <c r="B15" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C15" t="s">
-        <v>21</v>
+        <v>0.38714979988564885</v>
+      </c>
+      <c r="C15" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D15" t="s">
+        <v>21</v>
+      </c>
+      <c r="E15" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="2">
+      <c r="F15" s="3">
         <v>72500</v>
       </c>
-      <c r="F15" s="3">
+      <c r="G15" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G15" t="s">
-        <v>23</v>
-      </c>
       <c r="H15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" t="s">
         <v>35</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>44</v>
       </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>22</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>57</v>
       </c>
-      <c r="L15" s="2">
+      <c r="M15" s="3">
         <v>20000</v>
       </c>
-      <c r="M15" s="3">
+      <c r="N15" s="4">
         <v>0.343</v>
-      </c>
-      <c r="N15" s="4">
-        <v>0.38714979988564885</v>
       </c>
       <c r="O15" t="s">
         <v>58</v>
@@ -1595,13 +1595,13 @@
       <c r="P15" t="s">
         <v>59</v>
       </c>
-      <c r="Q15" s="1">
+      <c r="Q15" s="2">
         <v>46045.12805288195</v>
       </c>
-      <c r="R15" s="2">
+      <c r="R15" s="3">
         <v>45</v>
       </c>
-      <c r="S15" s="4">
+      <c r="S15" s="1">
         <v>0.27586206896551724</v>
       </c>
       <c r="T15" s="5">
@@ -1613,43 +1613,43 @@
         <v>20</v>
       </c>
       <c r="B16" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C16" t="s">
-        <v>21</v>
+        <v>0.38714979988564885</v>
+      </c>
+      <c r="C16" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D16" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" t="s">
         <v>22</v>
       </c>
-      <c r="E16" s="2">
+      <c r="F16" s="3">
         <v>72500</v>
       </c>
-      <c r="F16" s="3">
+      <c r="G16" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G16" t="s">
-        <v>23</v>
-      </c>
       <c r="H16" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" t="s">
         <v>35</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>44</v>
       </c>
-      <c r="J16" t="s">
+      <c r="K16" t="s">
         <v>22</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>57</v>
       </c>
-      <c r="L16" s="2">
+      <c r="M16" s="3">
         <v>20000</v>
       </c>
-      <c r="M16" s="3">
+      <c r="N16" s="4">
         <v>0.343</v>
-      </c>
-      <c r="N16" s="4">
-        <v>0.38714979988564885</v>
       </c>
       <c r="O16" t="s">
         <v>58</v>
@@ -1657,13 +1657,13 @@
       <c r="P16" t="s">
         <v>28</v>
       </c>
-      <c r="Q16" s="1">
+      <c r="Q16" s="2">
         <v>46045.1280428125</v>
       </c>
-      <c r="R16" s="2">
+      <c r="R16" s="3">
         <v>45</v>
       </c>
-      <c r="S16" s="4">
+      <c r="S16" s="1">
         <v>0.27586206896551724</v>
       </c>
       <c r="T16" s="5">
@@ -1675,43 +1675,43 @@
         <v>20</v>
       </c>
       <c r="B17" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C17" t="s">
-        <v>21</v>
+        <v>0.4139508290451686</v>
+      </c>
+      <c r="C17" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D17" t="s">
+        <v>21</v>
+      </c>
+      <c r="E17" t="s">
         <v>22</v>
       </c>
-      <c r="E17" s="2">
+      <c r="F17" s="3">
         <v>72500</v>
       </c>
-      <c r="F17" s="3">
+      <c r="G17" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G17" t="s">
-        <v>23</v>
-      </c>
       <c r="H17" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" t="s">
         <v>35</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>44</v>
       </c>
-      <c r="J17" t="s">
+      <c r="K17" t="s">
         <v>22</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>57</v>
       </c>
-      <c r="L17" s="2">
+      <c r="M17" s="3">
         <v>10000</v>
       </c>
-      <c r="M17" s="3">
+      <c r="N17" s="4">
         <v>0.328</v>
-      </c>
-      <c r="N17" s="4">
-        <v>0.4139508290451686</v>
       </c>
       <c r="O17" t="s">
         <v>58</v>
@@ -1719,13 +1719,13 @@
       <c r="P17" t="s">
         <v>28</v>
       </c>
-      <c r="Q17" s="1">
+      <c r="Q17" s="2">
         <v>46045.128032569446</v>
       </c>
-      <c r="R17" s="2">
+      <c r="R17" s="3">
         <v>45</v>
       </c>
-      <c r="S17" s="4">
+      <c r="S17" s="1">
         <v>0.13793103448275862</v>
       </c>
       <c r="T17" s="5">
@@ -1737,43 +1737,43 @@
         <v>20</v>
       </c>
       <c r="B18" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C18" t="s">
-        <v>21</v>
+        <v>-0.19617224880382786</v>
+      </c>
+      <c r="C18" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D18" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" t="s">
         <v>60</v>
       </c>
-      <c r="E18" s="2">
+      <c r="F18" s="3">
         <v>100000</v>
       </c>
-      <c r="F18" s="3">
+      <c r="G18" s="4">
         <v>0.00836</v>
       </c>
-      <c r="G18" t="s">
-        <v>23</v>
-      </c>
       <c r="H18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" t="s">
         <v>35</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>44</v>
       </c>
-      <c r="J18" t="s">
+      <c r="K18" t="s">
         <v>61</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>62</v>
       </c>
-      <c r="L18" s="2">
+      <c r="M18" s="3">
         <v>100000</v>
       </c>
-      <c r="M18" s="3">
+      <c r="N18" s="4">
         <v>0.01</v>
-      </c>
-      <c r="N18" s="4">
-        <v>-0.19617224880382786</v>
       </c>
       <c r="O18" t="s">
         <v>63</v>
@@ -1781,13 +1781,13 @@
       <c r="P18" t="s">
         <v>64</v>
       </c>
-      <c r="Q18" s="1">
+      <c r="Q18" s="2">
         <v>46044.1396249074</v>
       </c>
-      <c r="R18" s="2">
+      <c r="R18" s="3">
         <v>46</v>
       </c>
-      <c r="S18" s="4">
+      <c r="S18" s="1">
         <v>1</v>
       </c>
       <c r="T18" s="5">
@@ -1799,43 +1799,43 @@
         <v>20</v>
       </c>
       <c r="B19" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C19" t="s">
-        <v>21</v>
+        <v>0.07894736842105253</v>
+      </c>
+      <c r="C19" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D19" t="s">
+        <v>21</v>
+      </c>
+      <c r="E19" t="s">
         <v>60</v>
       </c>
-      <c r="E19" s="2">
+      <c r="F19" s="3">
         <v>100000</v>
       </c>
-      <c r="F19" s="3">
+      <c r="G19" s="4">
         <v>0.00836</v>
       </c>
-      <c r="G19" t="s">
-        <v>23</v>
-      </c>
       <c r="H19" t="s">
+        <v>23</v>
+      </c>
+      <c r="I19" t="s">
         <v>35</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>53</v>
       </c>
-      <c r="J19" t="s">
+      <c r="K19" t="s">
         <v>60</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>65</v>
       </c>
-      <c r="L19" s="2">
+      <c r="M19" s="3">
         <v>6000</v>
       </c>
-      <c r="M19" s="3">
+      <c r="N19" s="4">
         <v>0.0077</v>
-      </c>
-      <c r="N19" s="4">
-        <v>0.07894736842105253</v>
       </c>
       <c r="O19" t="s">
         <v>66</v>
@@ -1843,13 +1843,13 @@
       <c r="P19" t="s">
         <v>67</v>
       </c>
-      <c r="Q19" s="1">
+      <c r="Q19" s="2">
         <v>46044.139524432874</v>
       </c>
-      <c r="R19" s="2">
+      <c r="R19" s="3">
         <v>46</v>
       </c>
-      <c r="S19" s="4">
+      <c r="S19" s="1">
         <v>0.06</v>
       </c>
       <c r="T19" s="5">
@@ -1861,43 +1861,43 @@
         <v>20</v>
       </c>
       <c r="B20" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C20" t="s">
-        <v>21</v>
+        <v>0.07894736842105253</v>
+      </c>
+      <c r="C20" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D20" t="s">
+        <v>21</v>
+      </c>
+      <c r="E20" t="s">
         <v>60</v>
       </c>
-      <c r="E20" s="2">
+      <c r="F20" s="3">
         <v>100000</v>
       </c>
-      <c r="F20" s="3">
+      <c r="G20" s="4">
         <v>0.00836</v>
       </c>
-      <c r="G20" t="s">
-        <v>23</v>
-      </c>
       <c r="H20" t="s">
+        <v>23</v>
+      </c>
+      <c r="I20" t="s">
         <v>35</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>53</v>
       </c>
-      <c r="J20" t="s">
+      <c r="K20" t="s">
         <v>60</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>65</v>
       </c>
-      <c r="L20" s="2">
+      <c r="M20" s="3">
         <v>72000</v>
       </c>
-      <c r="M20" s="3">
+      <c r="N20" s="4">
         <v>0.0077</v>
-      </c>
-      <c r="N20" s="4">
-        <v>0.07894736842105253</v>
       </c>
       <c r="O20" t="s">
         <v>66</v>
@@ -1905,13 +1905,13 @@
       <c r="P20" t="s">
         <v>68</v>
       </c>
-      <c r="Q20" s="1">
+      <c r="Q20" s="2">
         <v>46044.13951418981</v>
       </c>
-      <c r="R20" s="2">
+      <c r="R20" s="3">
         <v>46</v>
       </c>
-      <c r="S20" s="4">
+      <c r="S20" s="1">
         <v>0.72</v>
       </c>
       <c r="T20" s="5">
@@ -1923,43 +1923,43 @@
         <v>20</v>
       </c>
       <c r="B21" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C21" t="s">
-        <v>21</v>
+        <v>0.41037735849056595</v>
+      </c>
+      <c r="C21" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D21" t="s">
+        <v>21</v>
+      </c>
+      <c r="E21" t="s">
         <v>22</v>
       </c>
-      <c r="E21" s="2">
+      <c r="F21" s="3">
         <v>72500</v>
       </c>
-      <c r="F21" s="3">
+      <c r="G21" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G21" t="s">
-        <v>23</v>
-      </c>
       <c r="H21" t="s">
+        <v>23</v>
+      </c>
+      <c r="I21" t="s">
         <v>35</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>53</v>
       </c>
-      <c r="J21" t="s">
+      <c r="K21" t="s">
         <v>22</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>69</v>
       </c>
-      <c r="L21" s="2">
+      <c r="M21" s="3">
         <v>20000</v>
       </c>
-      <c r="M21" s="3">
+      <c r="N21" s="4">
         <v>0.33</v>
-      </c>
-      <c r="N21" s="4">
-        <v>0.41037735849056595</v>
       </c>
       <c r="O21" t="s">
         <v>70</v>
@@ -1967,13 +1967,13 @@
       <c r="P21" t="s">
         <v>28</v>
       </c>
-      <c r="Q21" s="1">
+      <c r="Q21" s="2">
         <v>46031.23588373842</v>
       </c>
-      <c r="R21" s="2">
+      <c r="R21" s="3">
         <v>59</v>
       </c>
-      <c r="S21" s="4">
+      <c r="S21" s="1">
         <v>0.27586206896551724</v>
       </c>
       <c r="T21" s="5">
@@ -1985,43 +1985,43 @@
         <v>20</v>
       </c>
       <c r="B22" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C22" t="s">
-        <v>21</v>
+        <v>0.3785734705546026</v>
+      </c>
+      <c r="C22" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D22" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" t="s">
         <v>22</v>
       </c>
-      <c r="E22" s="2">
+      <c r="F22" s="3">
         <v>72500</v>
       </c>
-      <c r="F22" s="3">
+      <c r="G22" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G22" t="s">
-        <v>23</v>
-      </c>
       <c r="H22" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" t="s">
         <v>35</v>
       </c>
-      <c r="I22" t="s">
+      <c r="J22" t="s">
         <v>53</v>
       </c>
-      <c r="J22" t="s">
+      <c r="K22" t="s">
         <v>22</v>
       </c>
-      <c r="K22" t="s">
+      <c r="L22" t="s">
         <v>71</v>
       </c>
-      <c r="L22" s="2">
+      <c r="M22" s="3">
         <v>20000</v>
       </c>
-      <c r="M22" s="3">
+      <c r="N22" s="4">
         <v>0.3478</v>
-      </c>
-      <c r="N22" s="4">
-        <v>0.3785734705546026</v>
       </c>
       <c r="O22" t="s">
         <v>70</v>
@@ -2029,13 +2029,13 @@
       <c r="P22" t="s">
         <v>28</v>
       </c>
-      <c r="Q22" s="1">
+      <c r="Q22" s="2">
         <v>46031.235874108796</v>
       </c>
-      <c r="R22" s="2">
+      <c r="R22" s="3">
         <v>59</v>
       </c>
-      <c r="S22" s="4">
+      <c r="S22" s="1">
         <v>0.27586206896551724</v>
       </c>
       <c r="T22" s="5">
@@ -2047,43 +2047,43 @@
         <v>20</v>
       </c>
       <c r="B23" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C23" t="s">
-        <v>21</v>
+        <v>0.36106346483704976</v>
+      </c>
+      <c r="C23" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D23" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" t="s">
         <v>22</v>
       </c>
-      <c r="E23" s="2">
+      <c r="F23" s="3">
         <v>72500</v>
       </c>
-      <c r="F23" s="3">
+      <c r="G23" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G23" t="s">
-        <v>23</v>
-      </c>
       <c r="H23" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" t="s">
         <v>35</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>72</v>
       </c>
-      <c r="J23" t="s">
+      <c r="K23" t="s">
         <v>22</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>73</v>
       </c>
-      <c r="L23" s="2">
+      <c r="M23" s="3">
         <v>20000</v>
       </c>
-      <c r="M23" s="3">
+      <c r="N23" s="4">
         <v>0.3576</v>
-      </c>
-      <c r="N23" s="4">
-        <v>0.36106346483704976</v>
       </c>
       <c r="O23" t="s">
         <v>70</v>
@@ -2091,13 +2091,13 @@
       <c r="P23" t="s">
         <v>28</v>
       </c>
-      <c r="Q23" s="1">
+      <c r="Q23" s="2">
         <v>46031.23586418982</v>
       </c>
-      <c r="R23" s="2">
+      <c r="R23" s="3">
         <v>59</v>
       </c>
-      <c r="S23" s="4">
+      <c r="S23" s="1">
         <v>0.27586206896551724</v>
       </c>
       <c r="T23" s="5">
@@ -2109,43 +2109,43 @@
         <v>20</v>
       </c>
       <c r="B24" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C24" t="s">
-        <v>21</v>
+        <v>-0.06534090909090905</v>
+      </c>
+      <c r="C24" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D24" t="s">
+        <v>21</v>
+      </c>
+      <c r="E24" t="s">
         <v>52</v>
       </c>
-      <c r="E24" s="2">
+      <c r="F24" s="3">
         <v>84000</v>
       </c>
-      <c r="F24" s="3">
+      <c r="G24" s="4">
         <v>4.224</v>
       </c>
-      <c r="G24" t="s">
-        <v>23</v>
-      </c>
       <c r="H24" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" t="s">
         <v>35</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>53</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>52</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>54</v>
       </c>
-      <c r="L24" s="2">
+      <c r="M24" s="3">
         <v>56528</v>
       </c>
-      <c r="M24" s="3">
+      <c r="N24" s="4">
         <v>4.5</v>
-      </c>
-      <c r="N24" s="4">
-        <v>-0.06534090909090905</v>
       </c>
       <c r="O24" t="s">
         <v>74</v>
@@ -2153,13 +2153,13 @@
       <c r="P24" t="s">
         <v>75</v>
       </c>
-      <c r="Q24" s="1">
+      <c r="Q24" s="2">
         <v>46030.27382516203</v>
       </c>
-      <c r="R24" s="2">
+      <c r="R24" s="3">
         <v>60</v>
       </c>
-      <c r="S24" s="4">
+      <c r="S24" s="1">
         <v>0.672952380952381</v>
       </c>
       <c r="T24" s="5">
@@ -2171,43 +2171,43 @@
         <v>20</v>
       </c>
       <c r="B25" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C25" t="s">
-        <v>21</v>
+        <v>0.07989509440957893</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D25" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="2">
+      <c r="F25" s="3">
         <v>5400</v>
       </c>
-      <c r="F25" s="3">
+      <c r="G25" s="4">
         <v>14.67224</v>
       </c>
-      <c r="G25" t="s">
-        <v>23</v>
-      </c>
       <c r="H25" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" t="s">
         <v>35</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>53</v>
       </c>
-      <c r="J25" t="s">
+      <c r="K25" t="s">
         <v>76</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>69</v>
       </c>
-      <c r="L25" s="2">
+      <c r="M25" s="3">
         <v>1000</v>
       </c>
-      <c r="M25" s="3">
+      <c r="N25" s="4">
         <v>13.5</v>
-      </c>
-      <c r="N25" s="4">
-        <v>0.07989509440957893</v>
       </c>
       <c r="O25" t="s">
         <v>77</v>
@@ -2215,13 +2215,13 @@
       <c r="P25" t="s">
         <v>78</v>
       </c>
-      <c r="Q25" s="1">
+      <c r="Q25" s="2">
         <v>46030.273388182875</v>
       </c>
-      <c r="R25" s="2">
+      <c r="R25" s="3">
         <v>60</v>
       </c>
-      <c r="S25" s="4">
+      <c r="S25" s="1">
         <v>0.18518518518518517</v>
       </c>
       <c r="T25" s="5">
@@ -2233,43 +2233,43 @@
         <v>20</v>
       </c>
       <c r="B26" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C26" t="s">
-        <v>21</v>
+        <v>0.36106346483704976</v>
+      </c>
+      <c r="C26" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D26" t="s">
+        <v>21</v>
+      </c>
+      <c r="E26" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="2">
+      <c r="F26" s="3">
         <v>72500</v>
       </c>
-      <c r="F26" s="3">
+      <c r="G26" s="4">
         <v>0.55968</v>
       </c>
-      <c r="G26" t="s">
-        <v>23</v>
-      </c>
       <c r="H26" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" t="s">
         <v>35</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>72</v>
       </c>
-      <c r="J26" t="s">
+      <c r="K26" t="s">
         <v>22</v>
       </c>
-      <c r="K26" t="s">
+      <c r="L26" t="s">
         <v>73</v>
       </c>
-      <c r="L26" s="2">
+      <c r="M26" s="3">
         <v>20000</v>
       </c>
-      <c r="M26" s="3">
+      <c r="N26" s="4">
         <v>0.3576</v>
-      </c>
-      <c r="N26" s="4">
-        <v>0.36106346483704976</v>
       </c>
       <c r="O26" t="s">
         <v>70</v>
@@ -2277,13 +2277,13 @@
       <c r="P26" t="s">
         <v>28</v>
       </c>
-      <c r="Q26" s="1">
+      <c r="Q26" s="2">
         <v>46030.27282994213</v>
       </c>
-      <c r="R26" s="2">
+      <c r="R26" s="3">
         <v>60</v>
       </c>
-      <c r="S26" s="4">
+      <c r="S26" s="1">
         <v>0.27586206896551724</v>
       </c>
       <c r="T26" s="5">
@@ -2295,43 +2295,43 @@
         <v>20</v>
       </c>
       <c r="B27" s="1">
-        <v>46090.45766930556</v>
-      </c>
-      <c r="C27" t="s">
-        <v>21</v>
+        <v>-0.17442366246194013</v>
+      </c>
+      <c r="C27" s="2">
+        <v>46090.45766930556</v>
       </c>
       <c r="D27" t="s">
+        <v>21</v>
+      </c>
+      <c r="E27" t="s">
         <v>79</v>
       </c>
-      <c r="E27" s="2">
+      <c r="F27" s="3">
         <v>100000</v>
       </c>
-      <c r="F27" s="3">
+      <c r="G27" s="4">
         <v>0.004598</v>
       </c>
-      <c r="G27" t="s">
-        <v>23</v>
-      </c>
       <c r="H27" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" t="s">
         <v>35</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>53</v>
       </c>
-      <c r="J27" t="s">
+      <c r="K27" t="s">
         <v>79</v>
       </c>
-      <c r="K27" t="s">
+      <c r="L27" t="s">
         <v>65</v>
       </c>
-      <c r="L27" s="2">
+      <c r="M27" s="3">
         <v>15000</v>
       </c>
-      <c r="M27" s="3">
+      <c r="N27" s="4">
         <v>0.0054</v>
-      </c>
-      <c r="N27" s="4">
-        <v>-0.17442366246194013</v>
       </c>
       <c r="O27" t="s">
         <v>23</v>
@@ -2339,13 +2339,13 @@
       <c r="P27" t="s">
         <v>80</v>
       </c>
-      <c r="Q27" s="1">
+      <c r="Q27" s="2">
         <v>46029.223873587965</v>
       </c>
-      <c r="R27" s="2">
+      <c r="R27" s="3">
         <v>61</v>
       </c>
-      <c r="S27" s="4">
+      <c r="S27" s="1">
         <v>0.15</v>
       </c>
       <c r="T27" s="5">

</xml_diff>

<commit_message>
Leave MO Type blank for VQs (only applies to Market Offers)
Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trading Analysis/Vortex Matches/output/1130895_Good Prices.xlsx
+++ b/Trading Analysis/Vortex Matches/output/1130895_Good Prices.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="75">
   <si>
     <t>RFQ Number</t>
   </si>
@@ -121,9 +121,6 @@
     <t>VQ</t>
   </si>
   <si>
-    <t>Non-Traceable without Franchised lines</t>
-  </si>
-  <si>
     <t>Husky International</t>
   </si>
   <si>
@@ -136,18 +133,12 @@
     <t>FSM4JSMATR</t>
   </si>
   <si>
-    <t>Quality</t>
-  </si>
-  <si>
     <t>Flex-Com International Ltd</t>
   </si>
   <si>
     <t>13+</t>
   </si>
   <si>
-    <t>Suspended</t>
-  </si>
-  <si>
     <t>Elcom Components</t>
   </si>
   <si>
@@ -160,9 +151,6 @@
     <t>MPZ2012S101AT000</t>
   </si>
   <si>
-    <t>New/Ungraded Vendor</t>
-  </si>
-  <si>
     <t>Tencell LTD</t>
   </si>
   <si>
@@ -172,9 +160,6 @@
     <t>IMZA120R020M1H</t>
   </si>
   <si>
-    <t>Global Sourcing</t>
-  </si>
-  <si>
     <t>Tronix (HK) Ltd</t>
   </si>
   <si>
@@ -227,9 +212,6 @@
   </si>
   <si>
     <t>HK Firsttop Technology Ltd</t>
-  </si>
-  <si>
-    <t>Prohibited</t>
   </si>
   <si>
     <t>Esight International (HK) Ltd</t>
@@ -1079,13 +1061,13 @@
         <v>35</v>
       </c>
       <c r="J7" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="K7" t="s">
         <v>34</v>
       </c>
       <c r="L7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M7" s="3">
         <v>1906</v>
@@ -1094,10 +1076,10 @@
         <v>0.05</v>
       </c>
       <c r="O7" t="s">
+        <v>37</v>
+      </c>
+      <c r="P7" t="s">
         <v>38</v>
-      </c>
-      <c r="P7" t="s">
-        <v>39</v>
       </c>
       <c r="Q7" s="2">
         <v>46086.37278019676</v>
@@ -1126,7 +1108,7 @@
         <v>21</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F8" s="3">
         <v>24000</v>
@@ -1141,13 +1123,13 @@
         <v>35</v>
       </c>
       <c r="J8" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="K8" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" t="s">
         <v>40</v>
-      </c>
-      <c r="L8" t="s">
-        <v>42</v>
       </c>
       <c r="M8" s="3">
         <v>14400</v>
@@ -1156,10 +1138,10 @@
         <v>0.045</v>
       </c>
       <c r="O8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="Q8" s="2">
         <v>46086.355969791664</v>
@@ -1188,7 +1170,7 @@
         <v>21</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="3">
         <v>24000</v>
@@ -1203,13 +1185,13 @@
         <v>35</v>
       </c>
       <c r="J9" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="M9" s="3">
         <v>346</v>
@@ -1218,7 +1200,7 @@
         <v>0.07</v>
       </c>
       <c r="O9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P9" t="s">
         <v>23</v>
@@ -1265,13 +1247,13 @@
         <v>35</v>
       </c>
       <c r="J10" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="K10" t="s">
         <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="M10" s="3">
         <v>5677</v>
@@ -1280,10 +1262,10 @@
         <v>0.03</v>
       </c>
       <c r="O10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="Q10" s="2">
         <v>46086.35546523148</v>
@@ -1312,7 +1294,7 @@
         <v>21</v>
       </c>
       <c r="E11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F11" s="3">
         <v>3382</v>
@@ -1327,13 +1309,13 @@
         <v>35</v>
       </c>
       <c r="J11" t="s">
-        <v>49</v>
+        <v>23</v>
       </c>
       <c r="K11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="L11" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="M11" s="3">
         <v>8000</v>
@@ -1342,10 +1324,10 @@
         <v>0.00897</v>
       </c>
       <c r="O11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="P11" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="Q11" s="2">
         <v>46086.3509090625</v>
@@ -1374,7 +1356,7 @@
         <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F12" s="3">
         <v>84000</v>
@@ -1389,13 +1371,13 @@
         <v>35</v>
       </c>
       <c r="J12" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K12" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="L12" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M12" s="3">
         <v>84000</v>
@@ -1407,7 +1389,7 @@
         <v>23</v>
       </c>
       <c r="P12" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="Q12" s="2">
         <v>46085.228698402774</v>
@@ -1436,7 +1418,7 @@
         <v>21</v>
       </c>
       <c r="E13" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F13" s="3">
         <v>84000</v>
@@ -1451,13 +1433,13 @@
         <v>35</v>
       </c>
       <c r="J13" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K13" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="L13" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M13" s="3">
         <v>30000</v>
@@ -1469,7 +1451,7 @@
         <v>23</v>
       </c>
       <c r="P13" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="Q13" s="2">
         <v>46058.222427824076</v>
@@ -1513,13 +1495,13 @@
         <v>35</v>
       </c>
       <c r="J14" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K14" t="s">
         <v>22</v>
       </c>
       <c r="L14" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M14" s="3">
         <v>27500</v>
@@ -1528,7 +1510,7 @@
         <v>0.348</v>
       </c>
       <c r="O14" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="P14" t="s">
         <v>28</v>
@@ -1575,13 +1557,13 @@
         <v>35</v>
       </c>
       <c r="J15" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K15" t="s">
         <v>22</v>
       </c>
       <c r="L15" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M15" s="3">
         <v>20000</v>
@@ -1590,10 +1572,10 @@
         <v>0.343</v>
       </c>
       <c r="O15" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="P15" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="Q15" s="2">
         <v>46045.12805288195</v>
@@ -1637,13 +1619,13 @@
         <v>35</v>
       </c>
       <c r="J16" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K16" t="s">
         <v>22</v>
       </c>
       <c r="L16" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M16" s="3">
         <v>20000</v>
@@ -1652,7 +1634,7 @@
         <v>0.343</v>
       </c>
       <c r="O16" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="P16" t="s">
         <v>28</v>
@@ -1699,13 +1681,13 @@
         <v>35</v>
       </c>
       <c r="J17" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K17" t="s">
         <v>22</v>
       </c>
       <c r="L17" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="M17" s="3">
         <v>10000</v>
@@ -1714,7 +1696,7 @@
         <v>0.328</v>
       </c>
       <c r="O17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="P17" t="s">
         <v>28</v>
@@ -1746,7 +1728,7 @@
         <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F18" s="3">
         <v>100000</v>
@@ -1761,13 +1743,13 @@
         <v>35</v>
       </c>
       <c r="J18" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="K18" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="L18" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="M18" s="3">
         <v>100000</v>
@@ -1776,10 +1758,10 @@
         <v>0.01</v>
       </c>
       <c r="O18" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="P18" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="Q18" s="2">
         <v>46044.1396249074</v>
@@ -1808,7 +1790,7 @@
         <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F19" s="3">
         <v>100000</v>
@@ -1823,13 +1805,13 @@
         <v>35</v>
       </c>
       <c r="J19" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K19" t="s">
+        <v>55</v>
+      </c>
+      <c r="L19" t="s">
         <v>60</v>
-      </c>
-      <c r="L19" t="s">
-        <v>65</v>
       </c>
       <c r="M19" s="3">
         <v>6000</v>
@@ -1838,10 +1820,10 @@
         <v>0.0077</v>
       </c>
       <c r="O19" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="P19" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="Q19" s="2">
         <v>46044.139524432874</v>
@@ -1870,7 +1852,7 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="F20" s="3">
         <v>100000</v>
@@ -1885,13 +1867,13 @@
         <v>35</v>
       </c>
       <c r="J20" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K20" t="s">
+        <v>55</v>
+      </c>
+      <c r="L20" t="s">
         <v>60</v>
-      </c>
-      <c r="L20" t="s">
-        <v>65</v>
       </c>
       <c r="M20" s="3">
         <v>72000</v>
@@ -1900,10 +1882,10 @@
         <v>0.0077</v>
       </c>
       <c r="O20" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="P20" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="Q20" s="2">
         <v>46044.13951418981</v>
@@ -1947,13 +1929,13 @@
         <v>35</v>
       </c>
       <c r="J21" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K21" t="s">
         <v>22</v>
       </c>
       <c r="L21" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="M21" s="3">
         <v>20000</v>
@@ -1962,7 +1944,7 @@
         <v>0.33</v>
       </c>
       <c r="O21" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="P21" t="s">
         <v>28</v>
@@ -2009,13 +1991,13 @@
         <v>35</v>
       </c>
       <c r="J22" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K22" t="s">
         <v>22</v>
       </c>
       <c r="L22" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="M22" s="3">
         <v>20000</v>
@@ -2024,7 +2006,7 @@
         <v>0.3478</v>
       </c>
       <c r="O22" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="P22" t="s">
         <v>28</v>
@@ -2071,13 +2053,13 @@
         <v>35</v>
       </c>
       <c r="J23" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="K23" t="s">
         <v>22</v>
       </c>
       <c r="L23" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M23" s="3">
         <v>20000</v>
@@ -2086,7 +2068,7 @@
         <v>0.3576</v>
       </c>
       <c r="O23" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="P23" t="s">
         <v>28</v>
@@ -2118,7 +2100,7 @@
         <v>21</v>
       </c>
       <c r="E24" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F24" s="3">
         <v>84000</v>
@@ -2133,13 +2115,13 @@
         <v>35</v>
       </c>
       <c r="J24" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K24" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="L24" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="M24" s="3">
         <v>56528</v>
@@ -2148,10 +2130,10 @@
         <v>4.5</v>
       </c>
       <c r="O24" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="P24" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="Q24" s="2">
         <v>46030.27382516203</v>
@@ -2180,7 +2162,7 @@
         <v>21</v>
       </c>
       <c r="E25" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F25" s="3">
         <v>5400</v>
@@ -2195,13 +2177,13 @@
         <v>35</v>
       </c>
       <c r="J25" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K25" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="L25" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="M25" s="3">
         <v>1000</v>
@@ -2210,10 +2192,10 @@
         <v>13.5</v>
       </c>
       <c r="O25" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="P25" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="Q25" s="2">
         <v>46030.273388182875</v>
@@ -2257,13 +2239,13 @@
         <v>35</v>
       </c>
       <c r="J26" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="K26" t="s">
         <v>22</v>
       </c>
       <c r="L26" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="M26" s="3">
         <v>20000</v>
@@ -2272,7 +2254,7 @@
         <v>0.3576</v>
       </c>
       <c r="O26" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="P26" t="s">
         <v>28</v>
@@ -2304,7 +2286,7 @@
         <v>21</v>
       </c>
       <c r="E27" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="F27" s="3">
         <v>100000</v>
@@ -2319,13 +2301,13 @@
         <v>35</v>
       </c>
       <c r="J27" t="s">
-        <v>53</v>
+        <v>23</v>
       </c>
       <c r="K27" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="L27" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="M27" s="3">
         <v>15000</v>
@@ -2337,7 +2319,7 @@
         <v>23</v>
       </c>
       <c r="P27" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="Q27" s="2">
         <v>46029.223873587965</v>

</xml_diff>